<commit_message>
Clean up event schedule
</commit_message>
<xml_diff>
--- a/content/MotivateToSeattle/data/event-schedule.xlsx
+++ b/content/MotivateToSeattle/data/event-schedule.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10726"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BFE209D-30F9-CC48-80A5-33EAA4BE1829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="620" windowWidth="25520" windowHeight="26920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Event Schedule" state="visible" r:id="rId4"/>
+    <sheet name="Event Schedule" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
   <si>
     <t>Date</t>
   </si>
@@ -28,30 +32,15 @@
     <t>10/9/2026</t>
   </si>
   <si>
-    <t>1:00pm-5:00pm</t>
-  </si>
-  <si>
-    <t>Hilton Seattle Airport &amp; Conference Center</t>
-  </si>
-  <si>
-    <t>Set-Up (all dance halls)</t>
-  </si>
-  <si>
     <t>5:30pm-8:00pm</t>
   </si>
   <si>
-    <t>Hilton Seattle Airport &amp; Conference Center (Lobby)</t>
-  </si>
-  <si>
     <t>Registration</t>
   </si>
   <si>
     <t>6:30pm-7:00pm</t>
   </si>
   <si>
-    <t>Glacier</t>
-  </si>
-  <si>
     <t>GCA Caller slots (optional)</t>
   </si>
   <si>
@@ -85,29 +74,44 @@
     <t>Brunch (included in full registration)</t>
   </si>
   <si>
-    <t>2:00pm-3:00pm</t>
-  </si>
-  <si>
-    <t>Closing - All Headliners</t>
-  </si>
-  <si>
-    <t>3:00pm-4:00pm</t>
-  </si>
-  <si>
-    <t>Breakdown</t>
+    <t>9-12p</t>
+  </si>
+  <si>
+    <t>Glacier &amp; Horizon</t>
+  </si>
+  <si>
+    <t>All Halls</t>
+  </si>
+  <si>
+    <t>All level dancing</t>
+  </si>
+  <si>
+    <t>1-5p</t>
+  </si>
+  <si>
+    <t>11-2p</t>
+  </si>
+  <si>
+    <t>2-3p</t>
+  </si>
+  <si>
+    <t>Closing - All Headliens</t>
+  </si>
+  <si>
+    <t>Conference Center (Lobby)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -470,11 +474,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -488,7 +498,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -496,126 +506,134 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="D8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B9" t="s">
         <v>17</v>
       </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="D11" t="s">
         <v>26</v>
-      </c>
-      <c r="C10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restore missing Location values in Motivate to Seattle event schedule
A manual edit to event-schedule.xlsx (commit 8708308) left the Lunch
Break and Dinner Break rows without a Location, which the schedule
parser requires for every row — broke the production build for this
content set.
</commit_message>
<xml_diff>
--- a/content/MotivateToSeattle/data/event-schedule.xlsx
+++ b/content/MotivateToSeattle/data/event-schedule.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10726"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BFE209D-30F9-CC48-80A5-33EAA4BE1829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="25520" windowHeight="26920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="25520" windowHeight="26920"/>
   </bookViews>
   <sheets>
-    <sheet name="Event Schedule" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Event Schedule" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -35,12 +34,18 @@
     <t>5:30pm-8:00pm</t>
   </si>
   <si>
+    <t>Conference Center (Lobby)</t>
+  </si>
+  <si>
     <t>Registration</t>
   </si>
   <si>
     <t>6:30pm-7:00pm</t>
   </si>
   <si>
+    <t>Glacier &amp; Horizon</t>
+  </si>
+  <si>
     <t>GCA Caller slots (optional)</t>
   </si>
   <si>
@@ -53,9 +58,24 @@
     <t>10/10/2026</t>
   </si>
   <si>
+    <t>9-12p</t>
+  </si>
+  <si>
+    <t>All Halls</t>
+  </si>
+  <si>
+    <t>All level dancing</t>
+  </si>
+  <si>
+    <t>1-5p</t>
+  </si>
+  <si>
     <t>12:00pm-1:00pm</t>
   </si>
   <si>
+    <t>Hilton Seattle Airport &amp; Conference Center</t>
+  </si>
+  <si>
     <t>Lunch Break (on your own)</t>
   </si>
   <si>
@@ -74,21 +94,6 @@
     <t>Brunch (included in full registration)</t>
   </si>
   <si>
-    <t>9-12p</t>
-  </si>
-  <si>
-    <t>Glacier &amp; Horizon</t>
-  </si>
-  <si>
-    <t>All Halls</t>
-  </si>
-  <si>
-    <t>All level dancing</t>
-  </si>
-  <si>
-    <t>1-5p</t>
-  </si>
-  <si>
     <t>11-2p</t>
   </si>
   <si>
@@ -96,22 +101,19 @@
   </si>
   <si>
     <t>Closing - All Headliens</t>
-  </si>
-  <si>
-    <t>Conference Center (Lobby)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -474,17 +476,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
-    <col min="1" max="1" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -498,7 +500,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -506,134 +508,140 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
         <v>20</v>
       </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="D8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>23</v>
       </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="D9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>